<commit_message>
Initial commit - Automatic grading system
</commit_message>
<xml_diff>
--- a/data/question_model.xlsx
+++ b/data/question_model.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\19Feb1\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\2ndMarch\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A67EEB6-036E-4197-A11E-24B4D35EC69C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D58653B7-DCF3-46DA-BF54-649551912059}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DCE6906C-06BB-4A43-A67A-3D98AB49FD3F}"/>
   </bookViews>
@@ -132,102 +132,13 @@
     <t>model_answer</t>
   </si>
   <si>
-    <t>Explain the difference between compile-time polymorphism and runtime polymorphism in Java. Give examples for both.</t>
-  </si>
-  <si>
-    <t>Why are String objects immutable in Java? Explain with at least one advantage.</t>
-  </si>
-  <si>
-    <t>Explain how HashMap works internally in Java.</t>
-  </si>
-  <si>
-    <t>Explain the difference between checked exceptions and unchecked exceptions in Java with examples.</t>
-  </si>
-  <si>
-    <t>Explain the difference between Stack memory and Heap memory in Java.</t>
-  </si>
-  <si>
-    <t>Explain the difference between final, finally, and finalize in Java.</t>
-  </si>
-  <si>
-    <t>Explain the difference between multithreading and multiprocessing in Java.</t>
-  </si>
-  <si>
-    <t>Explain the architecture of JVM and its main components.</t>
-  </si>
-  <si>
-    <t>What is synchronization in Java? Why is it needed? Explain.</t>
-  </si>
-  <si>
-    <t>What is deadlock in Java? Explain how it occurs and give an example or situation.</t>
-  </si>
-  <si>
-    <t>What is Garbage Collection in Java? Explain how it works and why it is needed.</t>
-  </si>
-  <si>
-    <t>Explain the life cycle of a thread in Java.</t>
-  </si>
-  <si>
-    <t>Explain the difference between Callable and Runnable in Java.</t>
-  </si>
-  <si>
-    <t>Explain the difference between HashMap and ConcurrentHashMap in Java.</t>
-  </si>
-  <si>
     <t>What is the Executor Framework in Java? Why is it used?</t>
   </si>
   <si>
-    <t>What are Streams in Java 8? Explain their advantages.</t>
-  </si>
-  <si>
     <t>What is the volatile keyword in Java? Why is it used?</t>
   </si>
   <si>
     <t>What is serialization in Java? Why is it used?</t>
-  </si>
-  <si>
-    <t>What are Lambda expressions in Java 8? Explain their purpose and advantages.</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Explain the difference between </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>==</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> operator and </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>equals()</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> method in Java.</t>
-    </r>
   </si>
   <si>
     <r>
@@ -674,9 +585,6 @@
     <t>Concurrent programming involves managing multiple tasks that make progress independently, often sharing resources. Parallel programming executes multiple tasks simultaneously on multiple processors. Concurrency focuses on structure and responsiveness, while parallelism emphasizes performance and speed."</t>
   </si>
   <si>
-    <t>The Java Memory Model defines how threads interact through memory and specifies rules for reading and writing shared variables. It ensures consistency and visibility of data across threads. The model explains how changes made by one thread become visible to others and prevents unpredictable behavior in concurrent programs."</t>
-  </si>
-  <si>
     <t>A class loader is a component of the JVM responsible for loading class files into memory at runtime. It dynamically loads classes only when they are needed. Class loaders follow a hierarchical delegation model that improves security and prevents duplicate class loading."</t>
   </si>
   <si>
@@ -1217,42 +1125,24 @@
     <t>What is Java and why is it widely used?</t>
   </si>
   <si>
-    <t>Explain how Java achieves platform independence.</t>
-  </si>
-  <si>
     <t>What is the role of the JVM in Java?</t>
   </si>
   <si>
     <t>Differentiate between JDK, JRE, and JVM in detail.</t>
   </si>
   <si>
-    <t>Explain the Java program execution process step by step.</t>
-  </si>
-  <si>
     <t>What are the key features of Java and why are they important?</t>
   </si>
   <si>
     <t>What is object-oriented programming and how does Java implement it?</t>
   </si>
   <si>
-    <t>Explain the concept of a class and an object in Java.</t>
-  </si>
-  <si>
     <t>What is a constructor and why is it important?</t>
   </si>
   <si>
-    <t>Explain method overloading and overriding in Java.</t>
-  </si>
-  <si>
-    <t>Explain inheritance in Java and its advantages.</t>
-  </si>
-  <si>
     <t>What is encapsulation and why is it important in Java?</t>
   </si>
   <si>
-    <t>Explain polymorphism and its types in Java.</t>
-  </si>
-  <si>
     <t>What is abstraction and how is it implemented in Java?</t>
   </si>
   <si>
@@ -1295,9 +1185,6 @@
     <t>What is autoboxing and unboxing in Java?</t>
   </si>
   <si>
-    <t>Is Java pass-by-value or pass-by-reference? Explain.</t>
-  </si>
-  <si>
     <t>What is the static keyword in Java?</t>
   </si>
   <si>
@@ -1517,21 +1404,6 @@
     <t>What is the SOLID principle in Java design?</t>
   </si>
   <si>
-    <t>Explain the Single Responsibility Principle.</t>
-  </si>
-  <si>
-    <t>Explain the Open/Closed Principle.</t>
-  </si>
-  <si>
-    <t>Explain the Liskov Substitution Principle.</t>
-  </si>
-  <si>
-    <t>Explain the Interface Segregation Principle.</t>
-  </si>
-  <si>
-    <t>Explain the Dependency Inversion Principle.</t>
-  </si>
-  <si>
     <t>What is loose coupling in Java?</t>
   </si>
   <si>
@@ -1602,6 +1474,96 @@
   </si>
   <si>
     <t>What is a classpath in Java?</t>
+  </si>
+  <si>
+    <t>Discuss the difference between compile-time polymorphism and runtime polymorphism in Java. Give examples for both.</t>
+  </si>
+  <si>
+    <t>Why are String objects immutable in Java? Discuss with at least one advantage.</t>
+  </si>
+  <si>
+    <t>Discuss the difference between == operator and equals() method in Java.</t>
+  </si>
+  <si>
+    <t>Discuss how HashMap works internally in Java.</t>
+  </si>
+  <si>
+    <t>Discuss the difference between checked exceptions and unchecked exceptions in Java with examples.</t>
+  </si>
+  <si>
+    <t>Discuss the difference between Stack memory and Heap memory in Java.</t>
+  </si>
+  <si>
+    <t>Discuss the difference between final, finally, and finalize in Java.</t>
+  </si>
+  <si>
+    <t>Discuss the difference between multithreading and multiprocessing in Java.</t>
+  </si>
+  <si>
+    <t>Discuss the architecture of JVM and its main components.</t>
+  </si>
+  <si>
+    <t>What is synchronization in Java? Why is it needed? Discuss.</t>
+  </si>
+  <si>
+    <t>What is deadlock in Java? Discuss how it occurs and give an example or situation.</t>
+  </si>
+  <si>
+    <t>What is Garbage Collection in Java? Discuss how it works and why it is needed.</t>
+  </si>
+  <si>
+    <t>Discuss the life cycle of a thread in Java.</t>
+  </si>
+  <si>
+    <t>Discuss the difference between Callable and Runnable in Java.</t>
+  </si>
+  <si>
+    <t>Discuss the difference between HashMap and ConcurrentHashMap in Java.</t>
+  </si>
+  <si>
+    <t>What are Streams in Java 8? Discuss their advantages.</t>
+  </si>
+  <si>
+    <t>What are Lambda expressions in Java 8? Discuss their purpose and advantages.</t>
+  </si>
+  <si>
+    <t>Discuss how Java achieves platform independence.</t>
+  </si>
+  <si>
+    <t>Discuss the Java program execution process step by step.</t>
+  </si>
+  <si>
+    <t>Discuss the concept of a class and an object in Java.</t>
+  </si>
+  <si>
+    <t>Discuss method overloading and overriding in Java.</t>
+  </si>
+  <si>
+    <t>Discuss inheritance in Java and its advantages.</t>
+  </si>
+  <si>
+    <t>Discuss polymorphism and its types in Java.</t>
+  </si>
+  <si>
+    <t>Is Java pass-by-value or pass-by-reference? Discuss.</t>
+  </si>
+  <si>
+    <t>The Java Memory Model defines how threads interact through memory and specifies rules for reading and writing shared variables. It ensures consistency and visibility of data across threads. The model Discusss how changes made by one thread become visible to others and prevents unpredictable behavior in concurrent programs."</t>
+  </si>
+  <si>
+    <t>Discuss the Single Responsibility Principle.</t>
+  </si>
+  <si>
+    <t>Discuss the Open/Closed Principle.</t>
+  </si>
+  <si>
+    <t>Discuss the Liskov Substitution Principle.</t>
+  </si>
+  <si>
+    <t>Discuss the Interface Segregation Principle.</t>
+  </si>
+  <si>
+    <t>Discuss the Dependency Inversion Principle.</t>
   </si>
 </sst>
 </file>
@@ -2007,7 +1969,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>31</v>
+        <v>423</v>
       </c>
       <c r="C2" t="s">
         <v>22</v>
@@ -2018,7 +1980,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>32</v>
+        <v>424</v>
       </c>
       <c r="C3" t="s">
         <v>23</v>
@@ -2029,10 +1991,10 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>50</v>
+        <v>425</v>
       </c>
       <c r="C4" t="s">
-        <v>51</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -2040,10 +2002,10 @@
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>33</v>
+        <v>426</v>
       </c>
       <c r="C5" t="s">
-        <v>61</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -2051,7 +2013,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>34</v>
+        <v>427</v>
       </c>
       <c r="C6" t="s">
         <v>24</v>
@@ -2062,7 +2024,7 @@
         <v>7</v>
       </c>
       <c r="B7" t="s">
-        <v>35</v>
+        <v>428</v>
       </c>
       <c r="C7" t="s">
         <v>25</v>
@@ -2073,7 +2035,7 @@
         <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>36</v>
+        <v>429</v>
       </c>
       <c r="C8" t="s">
         <v>26</v>
@@ -2084,7 +2046,7 @@
         <v>9</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>37</v>
+        <v>430</v>
       </c>
       <c r="C9" t="s">
         <v>27</v>
@@ -2095,10 +2057,10 @@
         <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>38</v>
+        <v>431</v>
       </c>
       <c r="C10" t="s">
-        <v>52</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -2106,10 +2068,10 @@
         <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>39</v>
+        <v>432</v>
       </c>
       <c r="C11" t="s">
-        <v>53</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -2117,10 +2079,10 @@
         <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>40</v>
+        <v>433</v>
       </c>
       <c r="C12" t="s">
-        <v>54</v>
+        <v>37</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -2128,10 +2090,10 @@
         <v>13</v>
       </c>
       <c r="B13" t="s">
-        <v>41</v>
+        <v>434</v>
       </c>
       <c r="C13" t="s">
-        <v>55</v>
+        <v>38</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -2139,10 +2101,10 @@
         <v>14</v>
       </c>
       <c r="B14" t="s">
-        <v>42</v>
+        <v>435</v>
       </c>
       <c r="C14" t="s">
-        <v>56</v>
+        <v>39</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -2150,10 +2112,10 @@
         <v>15</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>43</v>
+        <v>436</v>
       </c>
       <c r="C15" t="s">
-        <v>62</v>
+        <v>45</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -2161,10 +2123,10 @@
         <v>16</v>
       </c>
       <c r="B16" t="s">
-        <v>44</v>
+        <v>437</v>
       </c>
       <c r="C16" t="s">
-        <v>57</v>
+        <v>40</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -2172,10 +2134,10 @@
         <v>17</v>
       </c>
       <c r="B17" t="s">
-        <v>45</v>
+        <v>31</v>
       </c>
       <c r="C17" t="s">
-        <v>58</v>
+        <v>41</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -2183,7 +2145,7 @@
         <v>18</v>
       </c>
       <c r="B18" t="s">
-        <v>46</v>
+        <v>438</v>
       </c>
       <c r="C18" t="s">
         <v>28</v>
@@ -2194,10 +2156,10 @@
         <v>19</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>47</v>
+        <v>32</v>
       </c>
       <c r="C19" t="s">
-        <v>59</v>
+        <v>42</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -2205,7 +2167,7 @@
         <v>20</v>
       </c>
       <c r="B20" t="s">
-        <v>48</v>
+        <v>33</v>
       </c>
       <c r="C20" t="s">
         <v>29</v>
@@ -2216,1479 +2178,1479 @@
         <v>21</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>49</v>
+        <v>439</v>
       </c>
       <c r="C21" t="s">
-        <v>60</v>
+        <v>43</v>
       </c>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" t="s">
-        <v>83</v>
+        <v>66</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>323</v>
+        <v>305</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>63</v>
+        <v>46</v>
       </c>
       <c r="D22" s="4"/>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" t="s">
-        <v>84</v>
+        <v>67</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>324</v>
+        <v>440</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>64</v>
+        <v>47</v>
       </c>
       <c r="D23" s="4"/>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" t="s">
-        <v>85</v>
+        <v>68</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>325</v>
+        <v>306</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>65</v>
+        <v>48</v>
       </c>
       <c r="D24" s="4"/>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" t="s">
-        <v>86</v>
+        <v>69</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>326</v>
+        <v>307</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>66</v>
+        <v>49</v>
       </c>
       <c r="D25" s="4"/>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" t="s">
-        <v>87</v>
+        <v>70</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>327</v>
+        <v>441</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>67</v>
+        <v>50</v>
       </c>
       <c r="D26" s="4"/>
     </row>
     <row r="27" spans="1:4">
       <c r="A27" t="s">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>328</v>
+        <v>308</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>68</v>
+        <v>51</v>
       </c>
       <c r="D27" s="4"/>
     </row>
     <row r="28" spans="1:4">
       <c r="A28" t="s">
-        <v>89</v>
+        <v>72</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>329</v>
+        <v>309</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>69</v>
+        <v>52</v>
       </c>
       <c r="D28" s="4"/>
     </row>
     <row r="29" spans="1:4">
       <c r="A29" t="s">
-        <v>90</v>
+        <v>73</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>330</v>
+        <v>442</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>70</v>
+        <v>53</v>
       </c>
       <c r="D29" s="4"/>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" t="s">
-        <v>91</v>
+        <v>74</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>331</v>
+        <v>310</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>71</v>
+        <v>54</v>
       </c>
       <c r="D30" s="4"/>
     </row>
     <row r="31" spans="1:4">
       <c r="A31" t="s">
-        <v>92</v>
+        <v>75</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>332</v>
+        <v>443</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>72</v>
+        <v>55</v>
       </c>
       <c r="D31" s="4"/>
     </row>
     <row r="32" spans="1:4">
       <c r="A32" t="s">
-        <v>93</v>
+        <v>76</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>333</v>
+        <v>444</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>73</v>
+        <v>56</v>
       </c>
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>94</v>
+        <v>77</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>334</v>
+        <v>311</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>74</v>
+        <v>57</v>
       </c>
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
-        <v>95</v>
+        <v>78</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>335</v>
+        <v>445</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>96</v>
+        <v>79</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>336</v>
+        <v>312</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>76</v>
+        <v>59</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
-        <v>97</v>
+        <v>80</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>337</v>
+        <v>313</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>98</v>
+        <v>81</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>338</v>
+        <v>314</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>78</v>
+        <v>61</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>99</v>
+        <v>82</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>339</v>
+        <v>315</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>79</v>
+        <v>62</v>
       </c>
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
-        <v>100</v>
+        <v>83</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>340</v>
+        <v>316</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>80</v>
+        <v>63</v>
       </c>
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
-        <v>101</v>
+        <v>84</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>341</v>
+        <v>317</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>81</v>
+        <v>64</v>
       </c>
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
-        <v>102</v>
+        <v>85</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>342</v>
+        <v>318</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>82</v>
+        <v>65</v>
       </c>
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
-        <v>183</v>
+        <v>165</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>343</v>
+        <v>319</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>103</v>
+        <v>86</v>
       </c>
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
-        <v>184</v>
+        <v>166</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>344</v>
+        <v>320</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>104</v>
+        <v>87</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>185</v>
+        <v>167</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>345</v>
+        <v>321</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>105</v>
+        <v>88</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>186</v>
+        <v>168</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>346</v>
+        <v>322</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>106</v>
+        <v>89</v>
       </c>
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>187</v>
+        <v>169</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>347</v>
+        <v>323</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>107</v>
+        <v>90</v>
       </c>
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>188</v>
+        <v>170</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>348</v>
+        <v>324</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>108</v>
+        <v>91</v>
       </c>
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
-        <v>189</v>
+        <v>171</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>349</v>
+        <v>325</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>109</v>
+        <v>92</v>
       </c>
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>190</v>
+        <v>172</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>350</v>
+        <v>446</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>110</v>
+        <v>93</v>
       </c>
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>191</v>
+        <v>173</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>351</v>
+        <v>326</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>111</v>
+        <v>94</v>
       </c>
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
-        <v>192</v>
+        <v>174</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>352</v>
+        <v>327</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>112</v>
+        <v>95</v>
       </c>
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
-        <v>193</v>
+        <v>175</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>353</v>
+        <v>328</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>113</v>
+        <v>96</v>
       </c>
     </row>
     <row r="53" spans="1:3">
       <c r="A53" t="s">
-        <v>194</v>
+        <v>176</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>354</v>
+        <v>329</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>114</v>
+        <v>97</v>
       </c>
     </row>
     <row r="54" spans="1:3">
       <c r="A54" t="s">
-        <v>195</v>
+        <v>177</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>355</v>
+        <v>330</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>115</v>
+        <v>98</v>
       </c>
     </row>
     <row r="55" spans="1:3">
       <c r="A55" t="s">
-        <v>196</v>
+        <v>178</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>356</v>
+        <v>331</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>116</v>
+        <v>99</v>
       </c>
     </row>
     <row r="56" spans="1:3">
       <c r="A56" t="s">
-        <v>197</v>
+        <v>179</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>357</v>
+        <v>332</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>117</v>
+        <v>100</v>
       </c>
     </row>
     <row r="57" spans="1:3">
       <c r="A57" t="s">
-        <v>198</v>
+        <v>180</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>358</v>
+        <v>333</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>118</v>
+        <v>101</v>
       </c>
     </row>
     <row r="58" spans="1:3">
       <c r="A58" t="s">
-        <v>199</v>
+        <v>181</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>359</v>
+        <v>334</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>119</v>
+        <v>102</v>
       </c>
     </row>
     <row r="59" spans="1:3">
       <c r="A59" t="s">
-        <v>200</v>
+        <v>182</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>360</v>
+        <v>335</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>120</v>
+        <v>103</v>
       </c>
     </row>
     <row r="60" spans="1:3">
       <c r="A60" t="s">
-        <v>201</v>
+        <v>183</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>361</v>
+        <v>336</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>121</v>
+        <v>104</v>
       </c>
     </row>
     <row r="61" spans="1:3">
       <c r="A61" t="s">
-        <v>202</v>
+        <v>184</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>362</v>
+        <v>337</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>122</v>
+        <v>105</v>
       </c>
     </row>
     <row r="62" spans="1:3">
       <c r="A62" t="s">
-        <v>203</v>
+        <v>185</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>363</v>
+        <v>338</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>123</v>
+        <v>106</v>
       </c>
     </row>
     <row r="63" spans="1:3">
       <c r="A63" t="s">
-        <v>204</v>
+        <v>186</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>364</v>
+        <v>339</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>124</v>
+        <v>107</v>
       </c>
     </row>
     <row r="64" spans="1:3">
       <c r="A64" t="s">
-        <v>205</v>
+        <v>187</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>365</v>
+        <v>340</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>125</v>
+        <v>108</v>
       </c>
     </row>
     <row r="65" spans="1:3">
       <c r="A65" t="s">
-        <v>206</v>
+        <v>188</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>366</v>
+        <v>341</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>126</v>
+        <v>109</v>
       </c>
     </row>
     <row r="66" spans="1:3">
       <c r="A66" t="s">
-        <v>207</v>
+        <v>189</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>367</v>
+        <v>342</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>127</v>
+        <v>110</v>
       </c>
     </row>
     <row r="67" spans="1:3">
       <c r="A67" t="s">
-        <v>208</v>
+        <v>190</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>368</v>
+        <v>343</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>128</v>
+        <v>111</v>
       </c>
     </row>
     <row r="68" spans="1:3">
       <c r="A68" t="s">
-        <v>209</v>
+        <v>191</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>369</v>
+        <v>344</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>129</v>
+        <v>112</v>
       </c>
     </row>
     <row r="69" spans="1:3">
       <c r="A69" t="s">
-        <v>210</v>
+        <v>192</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>370</v>
+        <v>345</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>130</v>
+        <v>113</v>
       </c>
     </row>
     <row r="70" spans="1:3">
       <c r="A70" t="s">
-        <v>211</v>
+        <v>193</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>371</v>
+        <v>346</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>131</v>
+        <v>114</v>
       </c>
     </row>
     <row r="71" spans="1:3">
       <c r="A71" t="s">
-        <v>212</v>
+        <v>194</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>372</v>
+        <v>347</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>132</v>
+        <v>115</v>
       </c>
     </row>
     <row r="72" spans="1:3">
       <c r="A72" t="s">
-        <v>213</v>
+        <v>195</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>373</v>
+        <v>348</v>
       </c>
       <c r="C72" s="3" t="s">
-        <v>133</v>
+        <v>116</v>
       </c>
     </row>
     <row r="73" spans="1:3">
       <c r="A73" t="s">
-        <v>214</v>
+        <v>196</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>374</v>
+        <v>349</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>134</v>
+        <v>117</v>
       </c>
     </row>
     <row r="74" spans="1:3">
       <c r="A74" t="s">
-        <v>215</v>
+        <v>197</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>375</v>
+        <v>350</v>
       </c>
       <c r="C74" s="3" t="s">
-        <v>135</v>
+        <v>118</v>
       </c>
     </row>
     <row r="75" spans="1:3">
       <c r="A75" t="s">
-        <v>216</v>
+        <v>198</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>376</v>
+        <v>351</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>136</v>
+        <v>119</v>
       </c>
     </row>
     <row r="76" spans="1:3">
       <c r="A76" t="s">
-        <v>217</v>
+        <v>199</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>377</v>
+        <v>352</v>
       </c>
       <c r="C76" s="3" t="s">
-        <v>137</v>
+        <v>120</v>
       </c>
     </row>
     <row r="77" spans="1:3">
       <c r="A77" t="s">
-        <v>218</v>
+        <v>200</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>378</v>
+        <v>353</v>
       </c>
       <c r="C77" s="3" t="s">
-        <v>138</v>
+        <v>121</v>
       </c>
     </row>
     <row r="78" spans="1:3">
       <c r="A78" t="s">
-        <v>219</v>
+        <v>201</v>
       </c>
       <c r="B78" s="3" t="s">
-        <v>379</v>
+        <v>354</v>
       </c>
       <c r="C78" s="3" t="s">
-        <v>139</v>
+        <v>122</v>
       </c>
     </row>
     <row r="79" spans="1:3">
       <c r="A79" t="s">
-        <v>220</v>
+        <v>202</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>380</v>
+        <v>355</v>
       </c>
       <c r="C79" s="3" t="s">
-        <v>140</v>
+        <v>123</v>
       </c>
     </row>
     <row r="80" spans="1:3">
       <c r="A80" t="s">
-        <v>221</v>
+        <v>203</v>
       </c>
       <c r="B80" s="3" t="s">
-        <v>381</v>
+        <v>356</v>
       </c>
       <c r="C80" s="3" t="s">
-        <v>141</v>
+        <v>124</v>
       </c>
     </row>
     <row r="81" spans="1:3">
       <c r="A81" t="s">
-        <v>222</v>
+        <v>204</v>
       </c>
       <c r="B81" s="3" t="s">
-        <v>382</v>
+        <v>357</v>
       </c>
       <c r="C81" s="3" t="s">
-        <v>142</v>
+        <v>125</v>
       </c>
     </row>
     <row r="82" spans="1:3">
       <c r="A82" t="s">
-        <v>223</v>
+        <v>205</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>383</v>
+        <v>358</v>
       </c>
       <c r="C82" s="3" t="s">
-        <v>143</v>
+        <v>447</v>
       </c>
     </row>
     <row r="83" spans="1:3">
       <c r="A83" t="s">
-        <v>224</v>
+        <v>206</v>
       </c>
       <c r="B83" s="3" t="s">
-        <v>384</v>
+        <v>359</v>
       </c>
       <c r="C83" s="3" t="s">
-        <v>144</v>
+        <v>126</v>
       </c>
     </row>
     <row r="84" spans="1:3">
       <c r="A84" t="s">
-        <v>225</v>
+        <v>207</v>
       </c>
       <c r="B84" s="3" t="s">
-        <v>385</v>
+        <v>360</v>
       </c>
       <c r="C84" s="3" t="s">
-        <v>145</v>
+        <v>127</v>
       </c>
     </row>
     <row r="85" spans="1:3">
       <c r="A85" t="s">
-        <v>226</v>
+        <v>208</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>386</v>
+        <v>361</v>
       </c>
       <c r="C85" s="3" t="s">
-        <v>146</v>
+        <v>128</v>
       </c>
     </row>
     <row r="86" spans="1:3">
       <c r="A86" t="s">
-        <v>227</v>
+        <v>209</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>387</v>
+        <v>362</v>
       </c>
       <c r="C86" s="3" t="s">
-        <v>147</v>
+        <v>129</v>
       </c>
     </row>
     <row r="87" spans="1:3">
       <c r="A87" t="s">
-        <v>228</v>
+        <v>210</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>388</v>
+        <v>363</v>
       </c>
       <c r="C87" s="3" t="s">
-        <v>148</v>
+        <v>130</v>
       </c>
     </row>
     <row r="88" spans="1:3">
       <c r="A88" t="s">
-        <v>229</v>
+        <v>211</v>
       </c>
       <c r="B88" s="3" t="s">
-        <v>389</v>
+        <v>364</v>
       </c>
       <c r="C88" s="3" t="s">
-        <v>149</v>
+        <v>131</v>
       </c>
     </row>
     <row r="89" spans="1:3">
       <c r="A89" t="s">
-        <v>230</v>
+        <v>212</v>
       </c>
       <c r="B89" s="3" t="s">
-        <v>390</v>
+        <v>365</v>
       </c>
       <c r="C89" s="3" t="s">
-        <v>150</v>
+        <v>132</v>
       </c>
     </row>
     <row r="90" spans="1:3">
       <c r="A90" t="s">
-        <v>231</v>
+        <v>213</v>
       </c>
       <c r="B90" s="3" t="s">
-        <v>391</v>
+        <v>366</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>151</v>
+        <v>133</v>
       </c>
     </row>
     <row r="91" spans="1:3">
       <c r="A91" t="s">
-        <v>232</v>
+        <v>214</v>
       </c>
       <c r="B91" s="3" t="s">
-        <v>392</v>
+        <v>367</v>
       </c>
       <c r="C91" s="3" t="s">
-        <v>152</v>
+        <v>134</v>
       </c>
     </row>
     <row r="92" spans="1:3">
       <c r="A92" t="s">
-        <v>233</v>
+        <v>215</v>
       </c>
       <c r="B92" s="3" t="s">
-        <v>393</v>
+        <v>368</v>
       </c>
       <c r="C92" s="3" t="s">
-        <v>153</v>
+        <v>135</v>
       </c>
     </row>
     <row r="93" spans="1:3">
       <c r="A93" t="s">
-        <v>234</v>
+        <v>216</v>
       </c>
       <c r="B93" s="3" t="s">
-        <v>394</v>
+        <v>369</v>
       </c>
       <c r="C93" s="3" t="s">
-        <v>154</v>
+        <v>136</v>
       </c>
     </row>
     <row r="94" spans="1:3">
       <c r="A94" t="s">
-        <v>235</v>
+        <v>217</v>
       </c>
       <c r="B94" s="3" t="s">
-        <v>395</v>
+        <v>370</v>
       </c>
       <c r="C94" s="3" t="s">
-        <v>155</v>
+        <v>137</v>
       </c>
     </row>
     <row r="95" spans="1:3">
       <c r="A95" t="s">
-        <v>236</v>
+        <v>218</v>
       </c>
       <c r="B95" s="3" t="s">
-        <v>396</v>
+        <v>371</v>
       </c>
       <c r="C95" s="3" t="s">
-        <v>156</v>
+        <v>138</v>
       </c>
     </row>
     <row r="96" spans="1:3">
       <c r="A96" t="s">
-        <v>237</v>
+        <v>219</v>
       </c>
       <c r="B96" s="3" t="s">
-        <v>397</v>
+        <v>372</v>
       </c>
       <c r="C96" s="3" t="s">
-        <v>157</v>
+        <v>139</v>
       </c>
     </row>
     <row r="97" spans="1:3">
       <c r="A97" t="s">
-        <v>238</v>
+        <v>220</v>
       </c>
       <c r="B97" s="3" t="s">
-        <v>398</v>
+        <v>373</v>
       </c>
       <c r="C97" s="3" t="s">
-        <v>158</v>
+        <v>140</v>
       </c>
     </row>
     <row r="98" spans="1:3">
       <c r="A98" t="s">
-        <v>239</v>
+        <v>221</v>
       </c>
       <c r="B98" s="3" t="s">
-        <v>399</v>
+        <v>374</v>
       </c>
       <c r="C98" s="3" t="s">
-        <v>159</v>
+        <v>141</v>
       </c>
     </row>
     <row r="99" spans="1:3">
       <c r="A99" t="s">
-        <v>240</v>
+        <v>222</v>
       </c>
       <c r="B99" s="3" t="s">
-        <v>400</v>
+        <v>375</v>
       </c>
       <c r="C99" s="3" t="s">
-        <v>160</v>
+        <v>142</v>
       </c>
     </row>
     <row r="100" spans="1:3">
       <c r="A100" t="s">
-        <v>241</v>
+        <v>223</v>
       </c>
       <c r="B100" s="3" t="s">
-        <v>401</v>
+        <v>376</v>
       </c>
       <c r="C100" s="3" t="s">
-        <v>161</v>
+        <v>143</v>
       </c>
     </row>
     <row r="101" spans="1:3">
       <c r="A101" t="s">
-        <v>242</v>
+        <v>224</v>
       </c>
       <c r="B101" s="3" t="s">
-        <v>402</v>
+        <v>377</v>
       </c>
       <c r="C101" s="3" t="s">
-        <v>162</v>
+        <v>144</v>
       </c>
     </row>
     <row r="102" spans="1:3">
       <c r="A102" t="s">
-        <v>243</v>
+        <v>225</v>
       </c>
       <c r="B102" s="3" t="s">
-        <v>403</v>
+        <v>378</v>
       </c>
       <c r="C102" s="3" t="s">
-        <v>163</v>
+        <v>145</v>
       </c>
     </row>
     <row r="103" spans="1:3">
       <c r="A103" t="s">
-        <v>244</v>
+        <v>226</v>
       </c>
       <c r="B103" s="3" t="s">
-        <v>404</v>
+        <v>379</v>
       </c>
       <c r="C103" s="3" t="s">
-        <v>164</v>
+        <v>146</v>
       </c>
     </row>
     <row r="104" spans="1:3">
       <c r="A104" t="s">
-        <v>245</v>
+        <v>227</v>
       </c>
       <c r="B104" s="3" t="s">
-        <v>405</v>
+        <v>380</v>
       </c>
       <c r="C104" s="3" t="s">
-        <v>165</v>
+        <v>147</v>
       </c>
     </row>
     <row r="105" spans="1:3">
       <c r="A105" t="s">
-        <v>246</v>
+        <v>228</v>
       </c>
       <c r="B105" s="3" t="s">
-        <v>406</v>
+        <v>381</v>
       </c>
       <c r="C105" s="3" t="s">
-        <v>166</v>
+        <v>148</v>
       </c>
     </row>
     <row r="106" spans="1:3">
       <c r="A106" t="s">
-        <v>247</v>
+        <v>229</v>
       </c>
       <c r="B106" s="3" t="s">
-        <v>407</v>
+        <v>382</v>
       </c>
       <c r="C106" s="3" t="s">
-        <v>167</v>
+        <v>149</v>
       </c>
     </row>
     <row r="107" spans="1:3">
       <c r="A107" t="s">
-        <v>248</v>
+        <v>230</v>
       </c>
       <c r="B107" s="3" t="s">
-        <v>408</v>
+        <v>383</v>
       </c>
       <c r="C107" s="3" t="s">
-        <v>168</v>
+        <v>150</v>
       </c>
     </row>
     <row r="108" spans="1:3">
       <c r="A108" t="s">
-        <v>249</v>
+        <v>231</v>
       </c>
       <c r="B108" s="3" t="s">
-        <v>409</v>
+        <v>384</v>
       </c>
       <c r="C108" s="3" t="s">
-        <v>169</v>
+        <v>151</v>
       </c>
     </row>
     <row r="109" spans="1:3">
       <c r="A109" t="s">
-        <v>250</v>
+        <v>232</v>
       </c>
       <c r="B109" s="3" t="s">
-        <v>410</v>
+        <v>385</v>
       </c>
       <c r="C109" s="3" t="s">
-        <v>170</v>
+        <v>152</v>
       </c>
     </row>
     <row r="110" spans="1:3">
       <c r="A110" t="s">
-        <v>251</v>
+        <v>233</v>
       </c>
       <c r="B110" s="3" t="s">
-        <v>411</v>
+        <v>386</v>
       </c>
       <c r="C110" s="3" t="s">
-        <v>171</v>
+        <v>153</v>
       </c>
     </row>
     <row r="111" spans="1:3">
       <c r="A111" t="s">
-        <v>252</v>
+        <v>234</v>
       </c>
       <c r="B111" s="3" t="s">
-        <v>412</v>
+        <v>387</v>
       </c>
       <c r="C111" s="3" t="s">
-        <v>172</v>
+        <v>154</v>
       </c>
     </row>
     <row r="112" spans="1:3">
       <c r="A112" t="s">
-        <v>253</v>
+        <v>235</v>
       </c>
       <c r="B112" s="3" t="s">
-        <v>413</v>
+        <v>388</v>
       </c>
       <c r="C112" s="3" t="s">
-        <v>173</v>
+        <v>155</v>
       </c>
     </row>
     <row r="113" spans="1:4">
       <c r="A113" t="s">
-        <v>254</v>
+        <v>236</v>
       </c>
       <c r="B113" s="3" t="s">
-        <v>414</v>
+        <v>389</v>
       </c>
       <c r="C113" s="3" t="s">
-        <v>174</v>
+        <v>156</v>
       </c>
     </row>
     <row r="114" spans="1:4">
       <c r="A114" t="s">
-        <v>255</v>
+        <v>237</v>
       </c>
       <c r="B114" s="3" t="s">
-        <v>415</v>
+        <v>390</v>
       </c>
       <c r="C114" s="3" t="s">
-        <v>175</v>
+        <v>157</v>
       </c>
     </row>
     <row r="115" spans="1:4">
       <c r="A115" t="s">
-        <v>256</v>
+        <v>238</v>
       </c>
       <c r="B115" s="3" t="s">
-        <v>416</v>
+        <v>391</v>
       </c>
       <c r="C115" s="3" t="s">
-        <v>176</v>
+        <v>158</v>
       </c>
     </row>
     <row r="116" spans="1:4">
       <c r="A116" t="s">
-        <v>257</v>
+        <v>239</v>
       </c>
       <c r="B116" s="3" t="s">
-        <v>417</v>
+        <v>392</v>
       </c>
       <c r="C116" s="3" t="s">
-        <v>177</v>
+        <v>159</v>
       </c>
     </row>
     <row r="117" spans="1:4">
       <c r="A117" t="s">
-        <v>258</v>
+        <v>240</v>
       </c>
       <c r="B117" s="3" t="s">
-        <v>418</v>
+        <v>393</v>
       </c>
       <c r="C117" s="3" t="s">
-        <v>178</v>
+        <v>160</v>
       </c>
     </row>
     <row r="118" spans="1:4">
       <c r="A118" t="s">
-        <v>259</v>
+        <v>241</v>
       </c>
       <c r="B118" s="3" t="s">
-        <v>419</v>
+        <v>394</v>
       </c>
       <c r="C118" s="3" t="s">
-        <v>179</v>
+        <v>161</v>
       </c>
     </row>
     <row r="119" spans="1:4">
       <c r="A119" t="s">
-        <v>260</v>
+        <v>242</v>
       </c>
       <c r="B119" s="3" t="s">
-        <v>420</v>
+        <v>395</v>
       </c>
       <c r="C119" s="3" t="s">
-        <v>180</v>
+        <v>162</v>
       </c>
     </row>
     <row r="120" spans="1:4">
       <c r="A120" t="s">
-        <v>261</v>
+        <v>243</v>
       </c>
       <c r="B120" s="3" t="s">
-        <v>421</v>
+        <v>396</v>
       </c>
       <c r="C120" s="3" t="s">
-        <v>181</v>
+        <v>163</v>
       </c>
     </row>
     <row r="121" spans="1:4">
       <c r="A121" t="s">
-        <v>262</v>
+        <v>244</v>
       </c>
       <c r="B121" s="3" t="s">
-        <v>422</v>
+        <v>397</v>
       </c>
       <c r="C121" s="3" t="s">
-        <v>182</v>
+        <v>164</v>
       </c>
     </row>
     <row r="122" spans="1:4">
       <c r="A122" t="s">
-        <v>263</v>
+        <v>245</v>
       </c>
       <c r="B122" s="3" t="s">
-        <v>423</v>
+        <v>398</v>
       </c>
       <c r="C122" s="3" t="s">
-        <v>293</v>
+        <v>275</v>
       </c>
       <c r="D122" s="4"/>
     </row>
     <row r="123" spans="1:4">
       <c r="A123" t="s">
-        <v>264</v>
+        <v>246</v>
       </c>
       <c r="B123" s="3" t="s">
-        <v>424</v>
+        <v>448</v>
       </c>
       <c r="C123" s="3" t="s">
-        <v>294</v>
+        <v>276</v>
       </c>
       <c r="D123" s="4"/>
     </row>
     <row r="124" spans="1:4">
       <c r="A124" t="s">
-        <v>265</v>
+        <v>247</v>
       </c>
       <c r="B124" s="3" t="s">
-        <v>425</v>
+        <v>449</v>
       </c>
       <c r="C124" s="3" t="s">
-        <v>295</v>
+        <v>277</v>
       </c>
       <c r="D124" s="4"/>
     </row>
     <row r="125" spans="1:4">
       <c r="A125" t="s">
-        <v>266</v>
+        <v>248</v>
       </c>
       <c r="B125" s="3" t="s">
-        <v>426</v>
+        <v>450</v>
       </c>
       <c r="C125" s="3" t="s">
-        <v>296</v>
+        <v>278</v>
       </c>
       <c r="D125" s="4"/>
     </row>
     <row r="126" spans="1:4">
       <c r="A126" t="s">
-        <v>267</v>
+        <v>249</v>
       </c>
       <c r="B126" s="3" t="s">
-        <v>427</v>
+        <v>451</v>
       </c>
       <c r="C126" s="3" t="s">
-        <v>297</v>
+        <v>279</v>
       </c>
       <c r="D126" s="4"/>
     </row>
     <row r="127" spans="1:4">
       <c r="A127" t="s">
-        <v>268</v>
+        <v>250</v>
       </c>
       <c r="B127" s="3" t="s">
-        <v>428</v>
+        <v>452</v>
       </c>
       <c r="C127" s="3" t="s">
-        <v>298</v>
+        <v>280</v>
       </c>
       <c r="D127" s="4"/>
     </row>
     <row r="128" spans="1:4">
       <c r="A128" t="s">
-        <v>269</v>
+        <v>251</v>
       </c>
       <c r="B128" s="3" t="s">
-        <v>429</v>
+        <v>399</v>
       </c>
       <c r="C128" s="3" t="s">
-        <v>299</v>
+        <v>281</v>
       </c>
       <c r="D128" s="4"/>
     </row>
     <row r="129" spans="1:4">
       <c r="A129" t="s">
-        <v>270</v>
+        <v>252</v>
       </c>
       <c r="B129" s="3" t="s">
-        <v>430</v>
+        <v>400</v>
       </c>
       <c r="C129" s="3" t="s">
-        <v>300</v>
+        <v>282</v>
       </c>
       <c r="D129" s="4"/>
     </row>
     <row r="130" spans="1:4">
       <c r="A130" t="s">
-        <v>271</v>
+        <v>253</v>
       </c>
       <c r="B130" s="3" t="s">
-        <v>431</v>
+        <v>401</v>
       </c>
       <c r="C130" s="3" t="s">
-        <v>301</v>
+        <v>283</v>
       </c>
       <c r="D130" s="4"/>
     </row>
     <row r="131" spans="1:4">
       <c r="A131" t="s">
-        <v>272</v>
+        <v>254</v>
       </c>
       <c r="B131" s="3" t="s">
-        <v>432</v>
+        <v>402</v>
       </c>
       <c r="C131" s="3" t="s">
-        <v>302</v>
+        <v>284</v>
       </c>
       <c r="D131" s="4"/>
     </row>
     <row r="132" spans="1:4">
       <c r="A132" t="s">
-        <v>273</v>
+        <v>255</v>
       </c>
       <c r="B132" s="3" t="s">
-        <v>433</v>
+        <v>403</v>
       </c>
       <c r="C132" s="3" t="s">
-        <v>303</v>
+        <v>285</v>
       </c>
       <c r="D132" s="4"/>
     </row>
     <row r="133" spans="1:4">
       <c r="A133" t="s">
-        <v>274</v>
+        <v>256</v>
       </c>
       <c r="B133" s="3" t="s">
-        <v>434</v>
+        <v>404</v>
       </c>
       <c r="C133" s="3" t="s">
-        <v>304</v>
+        <v>286</v>
       </c>
       <c r="D133" s="4"/>
     </row>
     <row r="134" spans="1:4">
       <c r="A134" t="s">
-        <v>275</v>
+        <v>257</v>
       </c>
       <c r="B134" s="3" t="s">
-        <v>435</v>
+        <v>405</v>
       </c>
       <c r="C134" s="3" t="s">
-        <v>305</v>
+        <v>287</v>
       </c>
       <c r="D134" s="4"/>
     </row>
     <row r="135" spans="1:4">
       <c r="A135" t="s">
-        <v>276</v>
+        <v>258</v>
       </c>
       <c r="B135" s="3" t="s">
-        <v>436</v>
+        <v>406</v>
       </c>
       <c r="C135" s="3" t="s">
-        <v>306</v>
+        <v>288</v>
       </c>
       <c r="D135" s="4"/>
     </row>
     <row r="136" spans="1:4">
       <c r="A136" t="s">
-        <v>277</v>
+        <v>259</v>
       </c>
       <c r="B136" s="3" t="s">
-        <v>437</v>
+        <v>407</v>
       </c>
       <c r="C136" s="3" t="s">
-        <v>307</v>
+        <v>289</v>
       </c>
       <c r="D136" s="4"/>
     </row>
     <row r="137" spans="1:4">
       <c r="A137" t="s">
-        <v>278</v>
+        <v>260</v>
       </c>
       <c r="B137" s="3" t="s">
-        <v>438</v>
+        <v>408</v>
       </c>
       <c r="C137" s="3" t="s">
-        <v>308</v>
+        <v>290</v>
       </c>
       <c r="D137" s="4"/>
     </row>
     <row r="138" spans="1:4">
       <c r="A138" t="s">
-        <v>279</v>
+        <v>261</v>
       </c>
       <c r="B138" s="3" t="s">
-        <v>439</v>
+        <v>409</v>
       </c>
       <c r="C138" s="3" t="s">
-        <v>309</v>
+        <v>291</v>
       </c>
       <c r="D138" s="4"/>
     </row>
     <row r="139" spans="1:4">
       <c r="A139" t="s">
-        <v>280</v>
+        <v>262</v>
       </c>
       <c r="B139" s="3" t="s">
-        <v>440</v>
+        <v>410</v>
       </c>
       <c r="C139" s="3" t="s">
-        <v>310</v>
+        <v>292</v>
       </c>
       <c r="D139" s="4"/>
     </row>
     <row r="140" spans="1:4">
       <c r="A140" t="s">
-        <v>281</v>
+        <v>263</v>
       </c>
       <c r="B140" s="3" t="s">
-        <v>441</v>
+        <v>411</v>
       </c>
       <c r="C140" s="3" t="s">
-        <v>311</v>
+        <v>293</v>
       </c>
       <c r="D140" s="4"/>
     </row>
     <row r="141" spans="1:4">
       <c r="A141" t="s">
-        <v>282</v>
+        <v>264</v>
       </c>
       <c r="B141" s="3" t="s">
-        <v>442</v>
+        <v>412</v>
       </c>
       <c r="C141" s="3" t="s">
-        <v>312</v>
+        <v>294</v>
       </c>
       <c r="D141" s="4"/>
     </row>
     <row r="142" spans="1:4">
       <c r="A142" t="s">
-        <v>283</v>
+        <v>265</v>
       </c>
       <c r="B142" s="3" t="s">
-        <v>443</v>
+        <v>413</v>
       </c>
       <c r="C142" s="3" t="s">
-        <v>313</v>
+        <v>295</v>
       </c>
       <c r="D142" s="4"/>
     </row>
     <row r="143" spans="1:4">
       <c r="A143" t="s">
-        <v>284</v>
+        <v>266</v>
       </c>
       <c r="B143" s="3" t="s">
-        <v>444</v>
+        <v>414</v>
       </c>
       <c r="C143" s="3" t="s">
-        <v>314</v>
+        <v>296</v>
       </c>
       <c r="D143" s="4"/>
     </row>
     <row r="144" spans="1:4">
       <c r="A144" t="s">
-        <v>285</v>
+        <v>267</v>
       </c>
       <c r="B144" s="3" t="s">
-        <v>445</v>
+        <v>415</v>
       </c>
       <c r="C144" s="3" t="s">
-        <v>315</v>
+        <v>297</v>
       </c>
       <c r="D144" s="4"/>
     </row>
     <row r="145" spans="1:4">
       <c r="A145" t="s">
-        <v>286</v>
+        <v>268</v>
       </c>
       <c r="B145" s="3" t="s">
-        <v>446</v>
+        <v>416</v>
       </c>
       <c r="C145" s="3" t="s">
-        <v>316</v>
+        <v>298</v>
       </c>
       <c r="D145" s="4"/>
     </row>
     <row r="146" spans="1:4">
       <c r="A146" t="s">
-        <v>287</v>
+        <v>269</v>
       </c>
       <c r="B146" s="3" t="s">
-        <v>447</v>
+        <v>417</v>
       </c>
       <c r="C146" s="3" t="s">
-        <v>317</v>
+        <v>299</v>
       </c>
       <c r="D146" s="4"/>
     </row>
     <row r="147" spans="1:4">
       <c r="A147" t="s">
-        <v>288</v>
+        <v>270</v>
       </c>
       <c r="B147" s="3" t="s">
-        <v>448</v>
+        <v>418</v>
       </c>
       <c r="C147" s="3" t="s">
-        <v>318</v>
+        <v>300</v>
       </c>
       <c r="D147" s="4"/>
     </row>
     <row r="148" spans="1:4">
       <c r="A148" t="s">
-        <v>289</v>
+        <v>271</v>
       </c>
       <c r="B148" s="3" t="s">
-        <v>449</v>
+        <v>419</v>
       </c>
       <c r="C148" s="3" t="s">
-        <v>319</v>
+        <v>301</v>
       </c>
       <c r="D148" s="4"/>
     </row>
     <row r="149" spans="1:4">
       <c r="A149" t="s">
-        <v>290</v>
+        <v>272</v>
       </c>
       <c r="B149" s="3" t="s">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="C149" s="3" t="s">
-        <v>320</v>
+        <v>302</v>
       </c>
       <c r="D149" s="4"/>
     </row>
     <row r="150" spans="1:4">
       <c r="A150" t="s">
-        <v>291</v>
+        <v>273</v>
       </c>
       <c r="B150" s="3" t="s">
-        <v>451</v>
+        <v>421</v>
       </c>
       <c r="C150" s="3" t="s">
-        <v>321</v>
+        <v>303</v>
       </c>
       <c r="D150" s="4"/>
     </row>
     <row r="151" spans="1:4">
       <c r="A151" t="s">
-        <v>292</v>
+        <v>274</v>
       </c>
       <c r="B151" s="3" t="s">
-        <v>452</v>
+        <v>422</v>
       </c>
       <c r="C151" s="3" t="s">
-        <v>322</v>
+        <v>304</v>
       </c>
       <c r="D151" s="4"/>
     </row>

</xml_diff>

<commit_message>
Add edit question feature with auto-translate Tamil/Hindi
</commit_message>
<xml_diff>
--- a/data/question_model.xlsx
+++ b/data/question_model.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\2ndMarch\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\25Mar\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D58653B7-DCF3-46DA-BF54-649551912059}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{039F67BA-D50A-4188-A84F-EE090E11D598}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DCE6906C-06BB-4A43-A67A-3D98AB49FD3F}"/>
   </bookViews>
@@ -100,10 +100,6 @@
   </si>
   <si>
     <t>Q020</t>
-  </si>
-  <si>
-    <t>Compile-time Polymorphism is achieved through Method Overloading. This happens when multiple methods share the same name but have different parameters. The compiler determines which method to call based on the method signature.
-Runtime Polymorphism is achieved through Method Overriding. This occurs when a subclass redefines a method that already exists in its parent class. The specific method to run is decided at runtime using dynamic binding, based on the actual object type.</t>
   </si>
   <si>
     <t>In Java, String objects are immutable, meaning their values cannot be changed once they are created. This immutability improves security, especially when Strings are used for sensitive data like passwords, and also enables memory optimization through the String Constant Pool.</t>
@@ -1476,94 +1472,98 @@
     <t>What is a classpath in Java?</t>
   </si>
   <si>
-    <t>Discuss the difference between compile-time polymorphism and runtime polymorphism in Java. Give examples for both.</t>
-  </si>
-  <si>
-    <t>Why are String objects immutable in Java? Discuss with at least one advantage.</t>
-  </si>
-  <si>
-    <t>Discuss the difference between == operator and equals() method in Java.</t>
-  </si>
-  <si>
-    <t>Discuss how HashMap works internally in Java.</t>
-  </si>
-  <si>
-    <t>Discuss the difference between checked exceptions and unchecked exceptions in Java with examples.</t>
-  </si>
-  <si>
-    <t>Discuss the difference between Stack memory and Heap memory in Java.</t>
-  </si>
-  <si>
-    <t>Discuss the difference between final, finally, and finalize in Java.</t>
-  </si>
-  <si>
-    <t>Discuss the difference between multithreading and multiprocessing in Java.</t>
-  </si>
-  <si>
-    <t>Discuss the architecture of JVM and its main components.</t>
-  </si>
-  <si>
-    <t>What is synchronization in Java? Why is it needed? Discuss.</t>
-  </si>
-  <si>
-    <t>What is deadlock in Java? Discuss how it occurs and give an example or situation.</t>
-  </si>
-  <si>
-    <t>What is Garbage Collection in Java? Discuss how it works and why it is needed.</t>
-  </si>
-  <si>
-    <t>Discuss the life cycle of a thread in Java.</t>
-  </si>
-  <si>
-    <t>Discuss the difference between Callable and Runnable in Java.</t>
-  </si>
-  <si>
-    <t>Discuss the difference between HashMap and ConcurrentHashMap in Java.</t>
-  </si>
-  <si>
-    <t>What are Streams in Java 8? Discuss their advantages.</t>
-  </si>
-  <si>
-    <t>What are Lambda expressions in Java 8? Discuss their purpose and advantages.</t>
-  </si>
-  <si>
-    <t>Discuss how Java achieves platform independence.</t>
-  </si>
-  <si>
-    <t>Discuss the Java program execution process step by step.</t>
-  </si>
-  <si>
-    <t>Discuss the concept of a class and an object in Java.</t>
-  </si>
-  <si>
-    <t>Discuss method overloading and overriding in Java.</t>
-  </si>
-  <si>
-    <t>Discuss inheritance in Java and its advantages.</t>
-  </si>
-  <si>
-    <t>Discuss polymorphism and its types in Java.</t>
-  </si>
-  <si>
-    <t>Is Java pass-by-value or pass-by-reference? Discuss.</t>
-  </si>
-  <si>
-    <t>The Java Memory Model defines how threads interact through memory and specifies rules for reading and writing shared variables. It ensures consistency and visibility of data across threads. The model Discusss how changes made by one thread become visible to others and prevents unpredictable behavior in concurrent programs."</t>
-  </si>
-  <si>
-    <t>Discuss the Single Responsibility Principle.</t>
-  </si>
-  <si>
-    <t>Discuss the Open/Closed Principle.</t>
-  </si>
-  <si>
-    <t>Discuss the Liskov Substitution Principle.</t>
-  </si>
-  <si>
-    <t>Discuss the Interface Segregation Principle.</t>
-  </si>
-  <si>
-    <t>Discuss the Dependency Inversion Principle.</t>
+    <t>State the difference between compile-time polymorphism and runtime polymorphism in Java. Give examples for both.</t>
+  </si>
+  <si>
+    <t>Why are String objects immutable in Java? State with at least one advantage.</t>
+  </si>
+  <si>
+    <t>State the difference between == operator and equals() method in Java.</t>
+  </si>
+  <si>
+    <t>State how HashMap works internally in Java.</t>
+  </si>
+  <si>
+    <t>State the difference between checked exceptions and unchecked exceptions in Java with examples.</t>
+  </si>
+  <si>
+    <t>State the difference between Stack memory and Heap memory in Java.</t>
+  </si>
+  <si>
+    <t>State the difference between final, finally, and finalize in Java.</t>
+  </si>
+  <si>
+    <t>State the difference between multithreading and multiprocessing in Java.</t>
+  </si>
+  <si>
+    <t>State the architecture of JVM and its main components.</t>
+  </si>
+  <si>
+    <t>What is synchronization in Java? Why is it needed? State.</t>
+  </si>
+  <si>
+    <t>What is deadlock in Java? State how it occurs and give an example or situation.</t>
+  </si>
+  <si>
+    <t>What is Garbage Collection in Java? State how it works and why it is needed.</t>
+  </si>
+  <si>
+    <t>State the life cycle of a thread in Java.</t>
+  </si>
+  <si>
+    <t>State the difference between Callable and Runnable in Java.</t>
+  </si>
+  <si>
+    <t>State the difference between HashMap and ConcurrentHashMap in Java.</t>
+  </si>
+  <si>
+    <t>What are Streams in Java 8? State their advantages.</t>
+  </si>
+  <si>
+    <t>What are Lambda expressions in Java 8? State their purpose and advantages.</t>
+  </si>
+  <si>
+    <t>State how Java achieves platform independence.</t>
+  </si>
+  <si>
+    <t>State the Java program execution process step by step.</t>
+  </si>
+  <si>
+    <t>State the concept of a class and an object in Java.</t>
+  </si>
+  <si>
+    <t>State method overloading and overriding in Java.</t>
+  </si>
+  <si>
+    <t>State inheritance in Java and its advantages.</t>
+  </si>
+  <si>
+    <t>State polymorphism and its types in Java.</t>
+  </si>
+  <si>
+    <t>Is Java pass-by-value or pass-by-reference? State.</t>
+  </si>
+  <si>
+    <t>The Java Memory Model defines how threads interact through memory and specifies rules for reading and writing shared variables. It ensures consistency and visibility of data across threads. The model States how changes made by one thread become visible to others and prevents unpredictable behavior in concurrent programs."</t>
+  </si>
+  <si>
+    <t>State the Single Responsibility Principle.</t>
+  </si>
+  <si>
+    <t>State the Open/Closed Principle.</t>
+  </si>
+  <si>
+    <t>State the Liskov Substitution Principle.</t>
+  </si>
+  <si>
+    <t>State the Interface Segregation Principle.</t>
+  </si>
+  <si>
+    <t>State the Dependency Inversion Principle.</t>
+  </si>
+  <si>
+    <t>Compile-time Polymorphism is achieved through Method Overloading. This happens when multiple methods share the same name but have different parameters. The compiler determines which method to call based on the method signature.
+Runtime Polymorphism is achieved through Method Overriding. This occurs when a subclass redefines a method that already exists in its parent class. The specific method to run is decided at runtime using dynamic binding, based on the actual object type.</t>
   </si>
 </sst>
 </file>
@@ -1621,7 +1621,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1633,6 +1633,7 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1961,7 +1962,7 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -1969,10 +1970,10 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>423</v>
-      </c>
-      <c r="C2" t="s">
-        <v>22</v>
+        <v>422</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>452</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1980,10 +1981,10 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="C3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1991,10 +1992,10 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="C4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -2002,10 +2003,10 @@
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="C5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -2013,10 +2014,10 @@
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="C6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -2024,10 +2025,10 @@
         <v>7</v>
       </c>
       <c r="B7" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="C7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -2035,10 +2036,10 @@
         <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="C8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -2046,10 +2047,10 @@
         <v>9</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="C9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -2057,10 +2058,10 @@
         <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="C10" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -2068,10 +2069,10 @@
         <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="C11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -2079,10 +2080,10 @@
         <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="C12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -2090,10 +2091,10 @@
         <v>13</v>
       </c>
       <c r="B13" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="C13" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -2101,10 +2102,10 @@
         <v>14</v>
       </c>
       <c r="B14" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="C14" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -2112,10 +2113,10 @@
         <v>15</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="C15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -2123,10 +2124,10 @@
         <v>16</v>
       </c>
       <c r="B16" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="C16" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -2134,10 +2135,10 @@
         <v>17</v>
       </c>
       <c r="B17" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C17" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -2145,10 +2146,10 @@
         <v>18</v>
       </c>
       <c r="B18" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="C18" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -2156,10 +2157,10 @@
         <v>19</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C19" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -2167,10 +2168,10 @@
         <v>20</v>
       </c>
       <c r="B20" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C20" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -2178,1479 +2179,1479 @@
         <v>21</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="C21" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D22" s="4"/>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D23" s="4"/>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D24" s="4"/>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D25" s="4"/>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D26" s="4"/>
     </row>
     <row r="27" spans="1:4">
       <c r="A27" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D27" s="4"/>
     </row>
     <row r="28" spans="1:4">
       <c r="A28" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D28" s="4"/>
     </row>
     <row r="29" spans="1:4">
       <c r="A29" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D29" s="4"/>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D30" s="4"/>
     </row>
     <row r="31" spans="1:4">
       <c r="A31" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D31" s="4"/>
     </row>
     <row r="32" spans="1:4">
       <c r="A32" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="53" spans="1:3">
       <c r="A53" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="54" spans="1:3">
       <c r="A54" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="55" spans="1:3">
       <c r="A55" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="56" spans="1:3">
       <c r="A56" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="57" spans="1:3">
       <c r="A57" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="58" spans="1:3">
       <c r="A58" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="59" spans="1:3">
       <c r="A59" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="60" spans="1:3">
       <c r="A60" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="61" spans="1:3">
       <c r="A61" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="62" spans="1:3">
       <c r="A62" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="63" spans="1:3">
       <c r="A63" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="64" spans="1:3">
       <c r="A64" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="65" spans="1:3">
       <c r="A65" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="66" spans="1:3">
       <c r="A66" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="67" spans="1:3">
       <c r="A67" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="68" spans="1:3">
       <c r="A68" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="69" spans="1:3">
       <c r="A69" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="70" spans="1:3">
       <c r="A70" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="71" spans="1:3">
       <c r="A71" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="72" spans="1:3">
       <c r="A72" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="C72" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="73" spans="1:3">
       <c r="A73" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="74" spans="1:3">
       <c r="A74" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="C74" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="75" spans="1:3">
       <c r="A75" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="76" spans="1:3">
       <c r="A76" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="C76" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="77" spans="1:3">
       <c r="A77" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C77" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="78" spans="1:3">
       <c r="A78" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B78" s="3" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C78" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="79" spans="1:3">
       <c r="A79" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="C79" s="3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="80" spans="1:3">
       <c r="A80" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B80" s="3" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C80" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="81" spans="1:3">
       <c r="A81" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B81" s="3" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="C81" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="82" spans="1:3">
       <c r="A82" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="C82" s="3" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="83" spans="1:3">
       <c r="A83" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B83" s="3" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C83" s="3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="84" spans="1:3">
       <c r="A84" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B84" s="3" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="C84" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="85" spans="1:3">
       <c r="A85" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="C85" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="86" spans="1:3">
       <c r="A86" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="C86" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="87" spans="1:3">
       <c r="A87" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="C87" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="88" spans="1:3">
       <c r="A88" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B88" s="3" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="C88" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="89" spans="1:3">
       <c r="A89" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B89" s="3" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="C89" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="90" spans="1:3">
       <c r="A90" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B90" s="3" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="91" spans="1:3">
       <c r="A91" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B91" s="3" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="C91" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="92" spans="1:3">
       <c r="A92" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B92" s="3" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="C92" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="93" spans="1:3">
       <c r="A93" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B93" s="3" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="C93" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="94" spans="1:3">
       <c r="A94" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B94" s="3" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="C94" s="3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="95" spans="1:3">
       <c r="A95" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B95" s="3" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="C95" s="3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="96" spans="1:3">
       <c r="A96" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B96" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="C96" s="3" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="97" spans="1:3">
       <c r="A97" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B97" s="3" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="C97" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="98" spans="1:3">
       <c r="A98" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B98" s="3" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="C98" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="99" spans="1:3">
       <c r="A99" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B99" s="3" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="C99" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="100" spans="1:3">
       <c r="A100" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B100" s="3" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C100" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="101" spans="1:3">
       <c r="A101" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B101" s="3" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="C101" s="3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="102" spans="1:3">
       <c r="A102" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B102" s="3" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="C102" s="3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="103" spans="1:3">
       <c r="A103" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B103" s="3" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="C103" s="3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="104" spans="1:3">
       <c r="A104" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B104" s="3" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="C104" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="105" spans="1:3">
       <c r="A105" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B105" s="3" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="C105" s="3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="106" spans="1:3">
       <c r="A106" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B106" s="3" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="C106" s="3" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="107" spans="1:3">
       <c r="A107" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B107" s="3" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="C107" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="108" spans="1:3">
       <c r="A108" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B108" s="3" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="C108" s="3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="109" spans="1:3">
       <c r="A109" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B109" s="3" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="C109" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="110" spans="1:3">
       <c r="A110" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B110" s="3" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="C110" s="3" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="111" spans="1:3">
       <c r="A111" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B111" s="3" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="C111" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="112" spans="1:3">
       <c r="A112" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B112" s="3" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="C112" s="3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="113" spans="1:4">
       <c r="A113" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B113" s="3" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="C113" s="3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="114" spans="1:4">
       <c r="A114" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B114" s="3" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="C114" s="3" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="115" spans="1:4">
       <c r="A115" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B115" s="3" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="C115" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="116" spans="1:4">
       <c r="A116" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B116" s="3" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="C116" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="117" spans="1:4">
       <c r="A117" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B117" s="3" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="C117" s="3" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="118" spans="1:4">
       <c r="A118" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B118" s="3" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="C118" s="3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="119" spans="1:4">
       <c r="A119" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B119" s="3" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="C119" s="3" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="120" spans="1:4">
       <c r="A120" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B120" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="C120" s="3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="121" spans="1:4">
       <c r="A121" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B121" s="3" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="C121" s="3" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="122" spans="1:4">
       <c r="A122" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B122" s="3" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="C122" s="3" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="D122" s="4"/>
     </row>
     <row r="123" spans="1:4">
       <c r="A123" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B123" s="3" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="C123" s="3" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="D123" s="4"/>
     </row>
     <row r="124" spans="1:4">
       <c r="A124" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B124" s="3" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="C124" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="D124" s="4"/>
     </row>
     <row r="125" spans="1:4">
       <c r="A125" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B125" s="3" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="C125" s="3" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="D125" s="4"/>
     </row>
     <row r="126" spans="1:4">
       <c r="A126" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B126" s="3" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="C126" s="3" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="D126" s="4"/>
     </row>
     <row r="127" spans="1:4">
       <c r="A127" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B127" s="3" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C127" s="3" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="D127" s="4"/>
     </row>
     <row r="128" spans="1:4">
       <c r="A128" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B128" s="3" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="C128" s="3" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="D128" s="4"/>
     </row>
     <row r="129" spans="1:4">
       <c r="A129" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B129" s="3" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="C129" s="3" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="D129" s="4"/>
     </row>
     <row r="130" spans="1:4">
       <c r="A130" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B130" s="3" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="C130" s="3" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="D130" s="4"/>
     </row>
     <row r="131" spans="1:4">
       <c r="A131" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B131" s="3" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="C131" s="3" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="D131" s="4"/>
     </row>
     <row r="132" spans="1:4">
       <c r="A132" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B132" s="3" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="C132" s="3" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="D132" s="4"/>
     </row>
     <row r="133" spans="1:4">
       <c r="A133" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B133" s="3" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="C133" s="3" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="D133" s="4"/>
     </row>
     <row r="134" spans="1:4">
       <c r="A134" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B134" s="3" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="C134" s="3" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="D134" s="4"/>
     </row>
     <row r="135" spans="1:4">
       <c r="A135" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B135" s="3" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="C135" s="3" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="D135" s="4"/>
     </row>
     <row r="136" spans="1:4">
       <c r="A136" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B136" s="3" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C136" s="3" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D136" s="4"/>
     </row>
     <row r="137" spans="1:4">
       <c r="A137" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B137" s="3" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="C137" s="3" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="D137" s="4"/>
     </row>
     <row r="138" spans="1:4">
       <c r="A138" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B138" s="3" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="C138" s="3" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="D138" s="4"/>
     </row>
     <row r="139" spans="1:4">
       <c r="A139" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B139" s="3" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="C139" s="3" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="D139" s="4"/>
     </row>
     <row r="140" spans="1:4">
       <c r="A140" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B140" s="3" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="C140" s="3" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="D140" s="4"/>
     </row>
     <row r="141" spans="1:4">
       <c r="A141" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B141" s="3" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="C141" s="3" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="D141" s="4"/>
     </row>
     <row r="142" spans="1:4">
       <c r="A142" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B142" s="3" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="C142" s="3" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="D142" s="4"/>
     </row>
     <row r="143" spans="1:4">
       <c r="A143" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B143" s="3" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="C143" s="3" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="D143" s="4"/>
     </row>
     <row r="144" spans="1:4">
       <c r="A144" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B144" s="3" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="C144" s="3" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="D144" s="4"/>
     </row>
     <row r="145" spans="1:4">
       <c r="A145" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B145" s="3" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="C145" s="3" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="D145" s="4"/>
     </row>
     <row r="146" spans="1:4">
       <c r="A146" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B146" s="3" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="C146" s="3" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D146" s="4"/>
     </row>
     <row r="147" spans="1:4">
       <c r="A147" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B147" s="3" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="C147" s="3" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="D147" s="4"/>
     </row>
     <row r="148" spans="1:4">
       <c r="A148" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B148" s="3" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="C148" s="3" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D148" s="4"/>
     </row>
     <row r="149" spans="1:4">
       <c r="A149" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B149" s="3" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="C149" s="3" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="D149" s="4"/>
     </row>
     <row r="150" spans="1:4">
       <c r="A150" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B150" s="3" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="C150" s="3" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="D150" s="4"/>
     </row>
     <row r="151" spans="1:4">
       <c r="A151" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B151" s="3" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="C151" s="3" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D151" s="4"/>
     </row>

</xml_diff>